<commit_message>
Sync banner library from Excel tables
</commit_message>
<xml_diff>
--- a/banners/01_Wuthering_Waves_confirmed.xlsx
+++ b/banners/01_Wuthering_Waves_confirmed.xlsx
@@ -2,26 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Banners" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Aptos"/>
-      <sz val="11"/>
-    </font>
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -33,8 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
-    <border/>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -44,7 +44,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -52,6 +52,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -412,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +467,33 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>1.19, 1.16, 1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3.7 Фаза 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1.7, 1.10, 1.11</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.41, 1.26, 1.24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin: update Wuthering Waves confirmed banners
</commit_message>
<xml_diff>
--- a/banners/01_Wuthering_Waves_confirmed.xlsx
+++ b/banners/01_Wuthering_Waves_confirmed.xlsx
@@ -65,33 +65,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.7 Фаза 1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-30</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-10-16</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.31, 1.32</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.19, 1.16, 1.9</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>